<commit_message>
done for applicability till 1st level
</commit_message>
<xml_diff>
--- a/Audit_Code/public/ISO27K1_2022_Compliance_Updated.xlsx
+++ b/Audit_Code/public/ISO27K1_2022_Compliance_Updated.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Compliance\Audit_Code\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23256" windowHeight="13176"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23250" windowHeight="13170"/>
   </bookViews>
   <sheets>
     <sheet name="Mandatory" sheetId="1" r:id="rId1"/>
@@ -13,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Mandatory!$A$1:$F$122</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="330">
   <si>
     <t>Context of the organization</t>
   </si>
@@ -1026,12 +1031,24 @@
   <si>
     <t>Nonconformity and corrective action</t>
   </si>
+  <si>
+    <t>Annex A</t>
+  </si>
+  <si>
+    <t>Organization Controls</t>
+  </si>
+  <si>
+    <t>Information security policy and topic-specific policies shall be defined, approved by management, published, communicated to and acknowledged by relevant personnel and relevant interested parties, and reviewed at planned intervals and if significant changes occur.</t>
+  </si>
+  <si>
+    <t>Information security roles and responsibilities shall be defined and allocated according to the organization needs.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1054,6 +1071,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -1094,7 +1117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1116,6 +1139,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1423,7 +1449,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1431,19 +1457,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F122"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F124"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="6" customWidth="1"/>
-    <col min="3" max="3" width="19.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="59.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="84.109375" style="6" customWidth="1"/>
-    <col min="7" max="16384" width="9.109375" style="6"/>
+    <col min="1" max="1" width="10.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="19.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="59.28515625" style="6" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="84.140625" style="6" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="3" t="s">
         <v>280</v>
@@ -1461,7 +1487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>4</v>
       </c>
@@ -1481,7 +1507,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>4</v>
       </c>
@@ -1501,7 +1527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>4</v>
       </c>
@@ -1521,7 +1547,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1541,7 +1567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -1561,7 +1587,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>4</v>
       </c>
@@ -1581,7 +1607,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>5</v>
       </c>
@@ -1601,7 +1627,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -1621,7 +1647,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>5</v>
       </c>
@@ -1641,7 +1667,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>5</v>
       </c>
@@ -1661,7 +1687,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>5</v>
       </c>
@@ -1681,7 +1707,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>5</v>
       </c>
@@ -1701,7 +1727,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>5</v>
       </c>
@@ -1721,7 +1747,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>5</v>
       </c>
@@ -1741,7 +1767,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>5</v>
       </c>
@@ -1761,7 +1787,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>5</v>
       </c>
@@ -1781,7 +1807,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>5</v>
       </c>
@@ -1801,7 +1827,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>5</v>
       </c>
@@ -1821,7 +1847,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>5</v>
       </c>
@@ -1841,7 +1867,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>5</v>
       </c>
@@ -1861,7 +1887,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <v>5</v>
       </c>
@@ -1881,7 +1907,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>5</v>
       </c>
@@ -1901,7 +1927,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
         <v>5</v>
       </c>
@@ -1921,7 +1947,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>6</v>
       </c>
@@ -1941,7 +1967,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
         <v>6</v>
       </c>
@@ -1961,7 +1987,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>6</v>
       </c>
@@ -1981,7 +2007,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <v>6</v>
       </c>
@@ -2001,7 +2027,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>6</v>
       </c>
@@ -2021,7 +2047,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
         <v>6</v>
       </c>
@@ -2041,7 +2067,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
         <v>6</v>
       </c>
@@ -2061,7 +2087,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <v>6</v>
       </c>
@@ -2081,7 +2107,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
         <v>6</v>
       </c>
@@ -2101,7 +2127,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
         <v>6</v>
       </c>
@@ -2121,7 +2147,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <v>6</v>
       </c>
@@ -2141,7 +2167,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
         <v>6</v>
       </c>
@@ -2161,7 +2187,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
         <v>6</v>
       </c>
@@ -2181,7 +2207,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
         <v>6</v>
       </c>
@@ -2201,7 +2227,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
         <v>6</v>
       </c>
@@ -2221,7 +2247,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
         <v>6</v>
       </c>
@@ -2241,7 +2267,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
         <v>6</v>
       </c>
@@ -2261,7 +2287,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
         <v>6</v>
       </c>
@@ -2281,7 +2307,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
         <v>6</v>
       </c>
@@ -2301,7 +2327,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
         <v>6</v>
       </c>
@@ -2321,7 +2347,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
         <v>6</v>
       </c>
@@ -2341,7 +2367,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
         <v>6</v>
       </c>
@@ -2361,7 +2387,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
         <v>6</v>
       </c>
@@ -2381,7 +2407,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
         <v>6</v>
       </c>
@@ -2401,7 +2427,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
         <v>6</v>
       </c>
@@ -2421,7 +2447,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
         <v>6</v>
       </c>
@@ -2441,7 +2467,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
         <v>6</v>
       </c>
@@ -2461,7 +2487,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
         <v>6</v>
       </c>
@@ -2481,7 +2507,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
         <v>6</v>
       </c>
@@ -2501,7 +2527,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
         <v>6</v>
       </c>
@@ -2521,7 +2547,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
         <v>6</v>
       </c>
@@ -2541,7 +2567,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
         <v>6</v>
       </c>
@@ -2561,7 +2587,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
         <v>6</v>
       </c>
@@ -2581,7 +2607,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
         <v>6</v>
       </c>
@@ -2601,7 +2627,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
         <v>7</v>
       </c>
@@ -2621,7 +2647,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
         <v>7</v>
       </c>
@@ -2641,7 +2667,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
         <v>7</v>
       </c>
@@ -2661,7 +2687,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <v>7</v>
       </c>
@@ -2681,7 +2707,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
         <v>7</v>
       </c>
@@ -2701,7 +2727,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
         <v>7</v>
       </c>
@@ -2721,7 +2747,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
         <v>7</v>
       </c>
@@ -2741,7 +2767,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="5">
         <v>7</v>
       </c>
@@ -2761,7 +2787,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="5">
         <v>7</v>
       </c>
@@ -2781,7 +2807,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="5">
         <v>7</v>
       </c>
@@ -2801,7 +2827,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="5">
         <v>7</v>
       </c>
@@ -2821,7 +2847,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="5">
         <v>7</v>
       </c>
@@ -2841,7 +2867,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="5">
         <v>7</v>
       </c>
@@ -2861,7 +2887,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="5">
         <v>7</v>
       </c>
@@ -2881,7 +2907,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="5">
         <v>7</v>
       </c>
@@ -2901,7 +2927,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="5">
         <v>7</v>
       </c>
@@ -2921,7 +2947,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="5">
         <v>7</v>
       </c>
@@ -2941,7 +2967,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="5">
         <v>7</v>
       </c>
@@ -2961,7 +2987,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="5">
         <v>7</v>
       </c>
@@ -2981,7 +3007,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="5">
         <v>7</v>
       </c>
@@ -3001,7 +3027,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="5">
         <v>7</v>
       </c>
@@ -3021,7 +3047,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="5">
         <v>7</v>
       </c>
@@ -3041,7 +3067,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="5">
         <v>7</v>
       </c>
@@ -3061,7 +3087,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="5">
         <v>8</v>
       </c>
@@ -3081,7 +3107,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="5">
         <v>8</v>
       </c>
@@ -3101,7 +3127,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="5">
         <v>8</v>
       </c>
@@ -3121,7 +3147,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="5">
         <v>8</v>
       </c>
@@ -3141,7 +3167,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="5">
         <v>8</v>
       </c>
@@ -3161,7 +3187,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="5">
         <v>8</v>
       </c>
@@ -3181,7 +3207,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="5">
         <v>9</v>
       </c>
@@ -3201,7 +3227,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="5">
         <v>9</v>
       </c>
@@ -3221,7 +3247,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="5">
         <v>9</v>
       </c>
@@ -3241,7 +3267,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="5">
         <v>9</v>
       </c>
@@ -3261,7 +3287,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="5">
         <v>9</v>
       </c>
@@ -3281,7 +3307,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="5">
         <v>9</v>
       </c>
@@ -3301,7 +3327,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="5">
         <v>9</v>
       </c>
@@ -3321,7 +3347,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="5">
         <v>9</v>
       </c>
@@ -3341,7 +3367,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="5">
         <v>9</v>
       </c>
@@ -3361,7 +3387,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="5">
         <v>9</v>
       </c>
@@ -3381,7 +3407,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="5">
         <v>9</v>
       </c>
@@ -3401,7 +3427,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="5">
         <v>9</v>
       </c>
@@ -3421,7 +3447,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="5">
         <v>9</v>
       </c>
@@ -3441,7 +3467,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="5">
         <v>9</v>
       </c>
@@ -3461,7 +3487,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="5">
         <v>9</v>
       </c>
@@ -3481,7 +3507,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="5">
         <v>9</v>
       </c>
@@ -3501,7 +3527,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="5">
         <v>9</v>
       </c>
@@ -3521,7 +3547,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="5">
         <v>9</v>
       </c>
@@ -3541,7 +3567,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="5">
         <v>9</v>
       </c>
@@ -3561,7 +3587,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="5">
         <v>9</v>
       </c>
@@ -3581,7 +3607,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="5">
         <v>9</v>
       </c>
@@ -3601,7 +3627,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="5">
         <v>9</v>
       </c>
@@ -3621,7 +3647,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="5">
         <v>9</v>
       </c>
@@ -3641,7 +3667,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="5">
         <v>9</v>
       </c>
@@ -3661,7 +3687,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="5">
         <v>10</v>
       </c>
@@ -3681,7 +3707,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="5">
         <v>10</v>
       </c>
@@ -3701,7 +3727,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="5">
         <v>10</v>
       </c>
@@ -3721,7 +3747,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="5">
         <v>10</v>
       </c>
@@ -3741,7 +3767,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="5">
         <v>10</v>
       </c>
@@ -3761,7 +3787,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="5">
         <v>10</v>
       </c>
@@ -3781,7 +3807,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="5">
         <v>10</v>
       </c>
@@ -3801,7 +3827,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="5">
         <v>10</v>
       </c>
@@ -3821,7 +3847,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="5">
         <v>10</v>
       </c>
@@ -3841,7 +3867,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="5">
         <v>10</v>
       </c>
@@ -3861,7 +3887,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="5">
         <v>10</v>
       </c>
@@ -3879,6 +3905,46 @@
       </c>
       <c r="F122" s="1" t="s">
         <v>279</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="57" x14ac:dyDescent="0.25">
+      <c r="A123" s="7">
+        <v>11</v>
+      </c>
+      <c r="B123" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C123" s="7">
+        <v>5</v>
+      </c>
+      <c r="D123" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="E123" s="7">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="F123" s="8" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A124" s="7">
+        <v>11</v>
+      </c>
+      <c r="B124" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C124" s="7">
+        <v>5</v>
+      </c>
+      <c r="D124" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="E124" s="7">
+        <v>5.2</v>
+      </c>
+      <c r="F124" s="6" t="s">
+        <v>329</v>
       </c>
     </row>
   </sheetData>
@@ -3891,13 +3957,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B122"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" style="7" customWidth="1"/>
-    <col min="2" max="2" width="68.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.42578125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>282</v>
       </c>
@@ -3905,7 +3971,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>4.0999999999999996</v>
       </c>
@@ -3913,7 +3979,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="str">
         <f>+MID(B3,1,3)</f>
         <v>4.2</v>
@@ -3922,7 +3988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="str">
         <f t="shared" ref="A4:A67" si="0">+MID(B4,1,3)</f>
         <v>4.2</v>
@@ -3931,7 +3997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="str">
         <f t="shared" si="0"/>
         <v>4.2</v>
@@ -3940,7 +4006,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="str">
         <f t="shared" si="0"/>
         <v>4.3</v>
@@ -3949,7 +4015,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="str">
         <f t="shared" si="0"/>
         <v>4.4</v>
@@ -3958,7 +4024,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -3967,7 +4033,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -3976,7 +4042,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -3985,7 +4051,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -3994,7 +4060,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -4003,7 +4069,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -4012,7 +4078,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -4021,7 +4087,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.1</v>
@@ -4030,7 +4096,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4039,7 +4105,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4048,7 +4114,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4057,7 +4123,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4066,7 +4132,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4075,7 +4141,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4084,7 +4150,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.2</v>
@@ -4093,7 +4159,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.3</v>
@@ -4102,7 +4168,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="str">
         <f t="shared" si="0"/>
         <v>5.3</v>
@@ -4111,7 +4177,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="str">
         <f>+MID(D25,1,3)</f>
         <v/>
@@ -4120,7 +4186,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="str">
         <f t="shared" ref="A26:A45" si="1">+MID(D26,1,3)</f>
         <v/>
@@ -4129,7 +4195,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4138,7 +4204,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4147,7 +4213,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4156,7 +4222,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4165,7 +4231,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4174,7 +4240,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4183,7 +4249,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4192,7 +4258,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4201,7 +4267,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4210,7 +4276,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4219,7 +4285,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4228,7 +4294,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4237,7 +4303,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4246,7 +4312,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4255,7 +4321,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4264,7 +4330,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4273,7 +4339,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4282,7 +4348,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4291,7 +4357,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4300,7 +4366,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4309,7 +4375,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4318,7 +4384,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4327,7 +4393,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4336,7 +4402,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4345,7 +4411,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4354,7 +4420,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4363,7 +4429,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4372,7 +4438,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4381,7 +4447,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4390,7 +4456,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4399,7 +4465,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.2</v>
@@ -4408,7 +4474,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="str">
         <f t="shared" si="0"/>
         <v>6.3</v>
@@ -4417,7 +4483,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.1</v>
@@ -4426,7 +4492,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.2</v>
@@ -4435,7 +4501,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.2</v>
@@ -4444,7 +4510,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.2</v>
@@ -4453,7 +4519,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.2</v>
@@ -4462,7 +4528,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.3</v>
@@ -4471,7 +4537,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.3</v>
@@ -4480,7 +4546,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.3</v>
@@ -4489,7 +4555,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="str">
         <f t="shared" si="0"/>
         <v>7.4</v>
@@ -4498,7 +4564,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="str">
         <f t="shared" ref="A68:A93" si="2">+MID(B68,1,3)</f>
         <v>7.4</v>
@@ -4507,7 +4573,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="str">
         <f t="shared" si="2"/>
         <v>7.4</v>
@@ -4516,7 +4582,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="str">
         <f t="shared" si="2"/>
         <v>7.4</v>
@@ -4525,7 +4591,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="str">
         <f>+MID(D71,1,3)</f>
         <v/>
@@ -4534,7 +4600,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="str">
         <f t="shared" ref="A72:A81" si="3">+MID(D72,1,3)</f>
         <v/>
@@ -4543,7 +4609,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4552,7 +4618,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4561,7 +4627,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4570,7 +4636,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4579,7 +4645,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4588,7 +4654,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4597,7 +4663,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4606,7 +4672,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4615,7 +4681,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -4624,7 +4690,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.1</v>
@@ -4633,7 +4699,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.1</v>
@@ -4642,7 +4708,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.1</v>
@@ -4651,7 +4717,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.1</v>
@@ -4660,7 +4726,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.2</v>
@@ -4669,7 +4735,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="str">
         <f t="shared" si="2"/>
         <v>8.3</v>
@@ -4678,7 +4744,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4687,7 +4753,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4696,7 +4762,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4705,7 +4771,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4714,7 +4780,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4723,7 +4789,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="str">
         <f t="shared" si="2"/>
         <v>9.1</v>
@@ -4732,169 +4798,169 @@
         <v>127</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="str">
-        <f>+MID(D94,1,3)</f>
+        <f t="shared" ref="A94:A100" si="4">+MID(D94,1,3)</f>
         <v/>
       </c>
       <c r="B94" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="str">
-        <f>+MID(D95,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B95" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="str">
-        <f>+MID(D96,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B96" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="str">
-        <f>+MID(D97,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B97" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="str">
-        <f>+MID(D98,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B98" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="str">
-        <f>+MID(D99,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B99" s="1" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="str">
-        <f>+MID(D100,1,3)</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="B100" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="str">
-        <f t="shared" ref="A101:A111" si="4">+MID(D101,1,3)</f>
+        <f t="shared" ref="A101:A111" si="5">+MID(D101,1,3)</f>
         <v/>
       </c>
       <c r="B101" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B102" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B103" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B104" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B105" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B106" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B107" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B108" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B109" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B110" s="1" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="B111" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="str">
         <f>+MID(B112,1,4)</f>
         <v>10.1</v>
@@ -4903,90 +4969,90 @@
         <v>157</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="str">
-        <f t="shared" ref="A113:A122" si="5">+MID(B113,1,4)</f>
+        <f t="shared" ref="A113:A122" si="6">+MID(B113,1,4)</f>
         <v>10.2</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>10.2</v>
       </c>
       <c r="B122" s="1" t="s">

</xml_diff>